<commit_message>
Add headlights, hero-showcase blocks, update importer
Automated migration updates generated by Experience Modernization Agent.

Changed files (15):
- blocks/headlights/_headlights.json
- blocks/headlights/headlights.css
- blocks/headlights/headlights.js
- blocks/headlights/metadata.json
- blocks/hero-showcase/hero-showcase.css
- component-definition.json
- component-filters.json
- component-models.json
- styles/styles.css
- tools/importer/import-homepage.bundle.js
- tools/importer/import-homepage.js
- tools/importer/page-templates.json
- tools/importer/parsers/headlights.js
- tools/importer/reports/import-homepage.report.xlsx
- tools/importer/reports/in/en/home.report.json
</commit_message>
<xml_diff>
--- a/tools/importer/reports/import-homepage.report.xlsx
+++ b/tools/importer/reports/import-homepage.report.xlsx
@@ -40,7 +40,7 @@
     <t>in/en/home.report.json</t>
   </si>
   <si>
-    <t>["hero-showcase","cards-dark","cards-dark","cards-dark","cards-dark","tabs-browse","carousel-legacy","columns-locate"]</t>
+    <t>["hero-showcase","headlights","headlights","cards-dark","cards-dark","cards-dark","tabs-browse","carousel-legacy","columns-locate"]</t>
   </si>
   <si>
     <t>in/en/home</t>
@@ -52,7 +52,7 @@
     <t>homepage</t>
   </si>
   <si>
-    <t>2026-04-06T14:04:55.973Z</t>
+    <t>2026-04-08T04:09:13.322Z</t>
   </si>
   <si>
     <t>Royal Enfield India | Roadster, Cruiser &amp; Adventure Bikes</t>

</xml_diff>